<commit_message>
fix: restrict task point calculation logic
Enforce strict rule that task points are only awarded to the creator or, in cross-team requests, to the officer who received the assignment if the creator is not an officer. Prevents inappropriate point allocation to supervisors.
</commit_message>
<xml_diff>
--- a/employee data.xlsx
+++ b/employee data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Walton\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Walton\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBFFCB08-E4B6-41F0-9906-0C1DA9498591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E903108-D6DB-4D4D-B5CD-84CB26688932}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="2625" windowWidth="29040" windowHeight="15720" xr2:uid="{22EE0D93-AB24-4600-95C8-184C655BE00F}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="159">
   <si>
     <t>ID</t>
   </si>
@@ -192,12 +192,6 @@
     <t>rac.rni.design-sd33@waltonplc.com</t>
   </si>
   <si>
-    <t>Md. Makfidunnabi</t>
-  </si>
-  <si>
-    <t>rac.rni.arnd1-t1@waltonplc.com</t>
-  </si>
-  <si>
     <t>Md. Alamgir Hossain</t>
   </si>
   <si>
@@ -213,27 +207,9 @@
     <t>ac.rni.design-eed10@waltonplc.com</t>
   </si>
   <si>
-    <t>Gazi Md. Safi Rayhan</t>
-  </si>
-  <si>
     <t>Senior Deputy Assistant Director</t>
   </si>
   <si>
-    <t>ac.rnd.design-sd7@waltonplc.com</t>
-  </si>
-  <si>
-    <t>Md. Mohibur Rahman</t>
-  </si>
-  <si>
-    <t>racrni.dar.simulation1@waltonplc.com</t>
-  </si>
-  <si>
-    <t>Shahiba Noshin</t>
-  </si>
-  <si>
-    <t>shahiba.noshin59018@waltonplc.com</t>
-  </si>
-  <si>
     <t>Md. Rashed Hossain</t>
   </si>
   <si>
@@ -390,12 +366,6 @@
     <t>Md. Lablue Islam</t>
   </si>
   <si>
-    <t>Md. Sabbir Hossen</t>
-  </si>
-  <si>
-    <t>Md. Assaduzzaman</t>
-  </si>
-  <si>
     <t>Md. Hamidur Rahman</t>
   </si>
   <si>
@@ -471,9 +441,6 @@
     <t>Proshenjit Chandra Barmon</t>
   </si>
   <si>
-    <t>Md. Khairul Kabeer</t>
-  </si>
-  <si>
     <t>Md. Atowar Rahman</t>
   </si>
   <si>
@@ -505,6 +472,45 @@
   </si>
   <si>
     <t>Technician</t>
+  </si>
+  <si>
+    <t>Md. Tanvir Rahman</t>
+  </si>
+  <si>
+    <t>Senior Executive Director</t>
+  </si>
+  <si>
+    <t>sajib@waltonplc.com</t>
+  </si>
+  <si>
+    <t>CBO</t>
+  </si>
+  <si>
+    <t>Shamim Ahmmed</t>
+  </si>
+  <si>
+    <t>Senior Additional Executive Director</t>
+  </si>
+  <si>
+    <t>shamim.ahmed@waltonplc.com</t>
+  </si>
+  <si>
+    <t>DCBO</t>
+  </si>
+  <si>
+    <t>Md. Nazmush Shakib Shahi</t>
+  </si>
+  <si>
+    <t>shahi69646@waltonplc.com</t>
+  </si>
+  <si>
+    <t>Md. Abdus Shakur</t>
+  </si>
+  <si>
+    <t>shakur69695@waltonplc.com</t>
+  </si>
+  <si>
+    <t>Md. Ashraful Haque</t>
   </si>
 </sst>
 </file>
@@ -514,7 +520,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="00000000000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -525,6 +531,13 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -534,7 +547,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -677,11 +690,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -725,8 +765,24 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1039,7 +1095,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B899631A-44BB-4936-AECC-854DA19530B8}">
-  <dimension ref="B1:G82"/>
+  <dimension ref="B1:G80"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="8.88671875" style="1"/>
@@ -1062,7 +1118,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>3</v>
@@ -1072,1542 +1128,1510 @@
       </c>
     </row>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B2" s="7">
-        <v>17668</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="8" t="s">
+      <c r="B2" s="15">
+        <v>1007</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>146</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="F2" s="17">
+        <v>1678028037</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="15">
+        <v>12467</v>
+      </c>
+      <c r="C3" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="F2" s="9">
-        <v>1678860396</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="7">
-        <v>19219</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="8" t="s">
+      <c r="D3" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="F3" s="9">
-        <v>1678860609</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>9</v>
+      <c r="E3" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="F3" s="17">
+        <v>1678048125</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" s="7">
-        <v>29766</v>
+        <v>17668</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>152</v>
+        <v>139</v>
       </c>
       <c r="F4" s="9">
-        <v>1678862217</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>12</v>
+        <v>1678860396</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="7">
-        <v>35866</v>
+        <v>19219</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F5" s="9">
-        <v>1678863942</v>
+        <v>1678860609</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="7">
-        <v>37091</v>
+        <v>29766</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="F6" s="9">
-        <v>1678860594</v>
+        <v>1678862217</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="7">
-        <v>38056</v>
+        <v>35866</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>14</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="F7" s="9">
-        <v>1678861735</v>
+        <v>1678863942</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="7">
-        <v>39301</v>
+        <v>37091</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="F8" s="9">
-        <v>1678862304</v>
+        <v>1678860594</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="7">
-        <v>41527</v>
+        <v>38056</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="F9" s="9">
-        <v>1678048167</v>
+        <v>1678861735</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="7">
-        <v>41053</v>
+        <v>39301</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="F10" s="9">
-        <v>1678048017</v>
+        <v>1678862304</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" s="7">
-        <v>43924</v>
+        <v>41527</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F11" s="9">
-        <v>1678864134</v>
+        <v>1678048167</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="7">
-        <v>45213</v>
+        <v>41053</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="F12" s="9">
-        <v>1678863107</v>
+        <v>1678048017</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="7">
-        <v>40760</v>
+        <v>43924</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F13" s="9">
-        <v>1678861127</v>
+        <v>1678864134</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="7">
-        <v>39766</v>
+        <v>45213</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F14" s="9">
-        <v>1678862835</v>
+        <v>1678863107</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="7">
-        <v>45064</v>
+        <v>40760</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>35</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F15" s="9">
-        <v>1678860540</v>
+        <v>1678861127</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="7">
-        <v>54589</v>
+        <v>39766</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>35</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="F16" s="9">
-        <v>1678862739</v>
+        <v>1678862835</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="7">
-        <v>50177</v>
+        <v>45064</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F17" s="9">
-        <v>1608985389</v>
+        <v>1678860540</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="7">
-        <v>41043</v>
+        <v>54589</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="F18" s="9">
-        <v>1678048007</v>
+        <v>1678862739</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="7">
-        <v>46419</v>
+        <v>50177</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>43</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F19" s="9">
-        <v>1608984875</v>
+        <v>1608985389</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="7">
-        <v>53127</v>
+        <v>41043</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F20" s="9">
-        <v>1608985621</v>
+        <v>1678048007</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="7">
-        <v>56742</v>
+        <v>46419</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F21" s="9">
-        <v>1608985488</v>
+        <v>1608984875</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="7">
-        <v>5101</v>
+        <v>53127</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F22" s="9">
-        <v>1686695257</v>
+        <v>1608985621</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="7">
-        <v>57772</v>
+        <v>5101</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F23" s="9">
-        <v>1678861684</v>
+        <v>1686695257</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="7">
-        <v>58595</v>
+        <v>57772</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F24" s="9">
-        <v>1678860486</v>
+        <v>1678861684</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B25" s="7">
-        <v>58640</v>
+        <v>66063</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F25" s="9">
-        <v>1608985215</v>
+        <v>1678860528</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="7">
-        <v>59018</v>
+        <v>68016</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F26" s="9">
-        <v>1608985816</v>
+        <v>1678864119</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B27" s="7">
-        <v>66063</v>
+        <v>39823</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F27" s="9">
-        <v>1678860528</v>
+        <v>1678863068</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B28" s="7">
-        <v>68016</v>
+        <v>69646</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>68</v>
+        <v>154</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F28" s="9">
-        <v>1678864119</v>
+        <v>1686695525</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>69</v>
+        <v>155</v>
       </c>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B29" s="7">
-        <v>39823</v>
+        <v>69695</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>70</v>
+        <v>156</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="F29" s="9">
-        <v>1678863068</v>
-      </c>
-      <c r="G29" s="10" t="s">
-        <v>72</v>
+        <v>1678863759</v>
+      </c>
+      <c r="G29" s="19" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B30" s="7">
-        <v>19359</v>
+        <v>69810</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>73</v>
+        <v>158</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="F30" s="9">
-        <v>1686695523</v>
-      </c>
-      <c r="G30" s="10" t="s">
-        <v>75</v>
+        <v>1522127684</v>
+      </c>
+      <c r="G30" s="19" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="7">
-        <v>19348</v>
+        <v>19359</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="F31" s="9">
-        <v>1678860916</v>
+        <v>1686695523</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="7">
-        <v>42949</v>
+        <v>19348</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="F32" s="9">
-        <v>1678862906</v>
+        <v>1678860916</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B33" s="7">
-        <v>4461</v>
+        <v>42949</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="F33" s="9">
-        <v>1678048246</v>
+        <v>1678862906</v>
       </c>
       <c r="G33" s="10" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B34" s="7">
-        <v>58175</v>
+        <v>4461</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="F34" s="9">
-        <v>1608984816</v>
+        <v>1678048246</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B35" s="7">
-        <v>38250</v>
+        <v>58175</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="F35" s="9">
-        <v>1678861825</v>
+        <v>1608984816</v>
       </c>
       <c r="G35" s="10" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B36" s="7">
-        <v>67123</v>
+        <v>38250</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="F36" s="9">
-        <v>1608985078</v>
+        <v>1678861825</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B37" s="7">
-        <v>41412</v>
+        <v>67123</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="F37" s="9">
-        <v>1686695196</v>
+        <v>1608985078</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
     </row>
     <row r="38" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B38" s="7">
-        <v>39939</v>
+        <v>41412</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="F38" s="9">
-        <v>1678860136</v>
+        <v>1686695196</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B39" s="7">
-        <v>7669</v>
+        <v>39939</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="F39" s="9">
-        <v>1686695403</v>
+        <v>1678860136</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
     </row>
     <row r="40" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B40" s="7">
-        <v>6810</v>
+        <v>7669</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="F40" s="9">
-        <v>1678861505</v>
-      </c>
-      <c r="G40" s="10"/>
+        <v>1686695403</v>
+      </c>
+      <c r="G40" s="10" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B41" s="7">
-        <v>21527</v>
+        <v>6810</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F41" s="9">
-        <v>1678862342</v>
+        <v>1678861505</v>
       </c>
       <c r="G41" s="10"/>
     </row>
     <row r="42" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B42" s="7">
-        <v>30644</v>
+        <v>21527</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F42" s="9">
-        <v>1678861417</v>
+        <v>1678862342</v>
       </c>
       <c r="G42" s="10"/>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B43" s="7">
-        <v>22760</v>
+        <v>30644</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F43" s="9">
-        <v>1686695894</v>
+        <v>1678861417</v>
       </c>
       <c r="G43" s="10"/>
     </row>
     <row r="44" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B44" s="7">
-        <v>20368</v>
+        <v>22760</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F44" s="9">
-        <v>1678861251</v>
+        <v>1686695894</v>
       </c>
       <c r="G44" s="10"/>
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B45" s="7">
-        <v>45660</v>
+        <v>20368</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F45" s="9">
-        <v>1686695599</v>
+        <v>1678861251</v>
       </c>
       <c r="G45" s="10"/>
     </row>
     <row r="46" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B46" s="7">
-        <v>48309</v>
+        <v>45660</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F46" s="9">
-        <v>1608984739</v>
+        <v>1686695599</v>
       </c>
       <c r="G46" s="10"/>
     </row>
     <row r="47" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B47" s="7">
-        <v>48566</v>
+        <v>48309</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F47" s="9">
-        <v>1678862664</v>
+        <v>1608984739</v>
       </c>
       <c r="G47" s="10"/>
     </row>
     <row r="48" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B48" s="7">
-        <v>52903</v>
+        <v>48566</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F48" s="9">
-        <v>1608985677</v>
+        <v>1678862664</v>
       </c>
       <c r="G48" s="10"/>
     </row>
     <row r="49" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B49" s="7">
-        <v>37413</v>
+        <v>52903</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F49" s="9">
-        <v>1678862982</v>
+        <v>1608985677</v>
       </c>
       <c r="G49" s="10"/>
     </row>
     <row r="50" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B50" s="7">
-        <v>40664</v>
+        <v>37413</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F50" s="9">
-        <v>1678861519</v>
+        <v>1678862982</v>
       </c>
       <c r="G50" s="10"/>
     </row>
     <row r="51" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B51" s="7">
-        <v>42234</v>
+        <v>40664</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F51" s="9">
-        <v>1678862521</v>
+        <v>1678861519</v>
       </c>
       <c r="G51" s="10"/>
     </row>
     <row r="52" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B52" s="7">
-        <v>42274</v>
+        <v>42234</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F52" s="9">
-        <v>1686695162</v>
+        <v>1678862521</v>
       </c>
       <c r="G52" s="10"/>
     </row>
     <row r="53" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B53" s="7">
-        <v>43081</v>
+        <v>42274</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F53" s="9">
-        <v>1678864219</v>
+        <v>1686695162</v>
       </c>
       <c r="G53" s="10"/>
     </row>
     <row r="54" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B54" s="7">
-        <v>44415</v>
+        <v>43081</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F54" s="9">
-        <v>1678860819</v>
+        <v>1678864219</v>
       </c>
       <c r="G54" s="10"/>
     </row>
     <row r="55" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B55" s="7">
-        <v>56489</v>
+        <v>44415</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F55" s="9">
-        <v>1608984973</v>
+        <v>1678860819</v>
       </c>
       <c r="G55" s="10"/>
     </row>
     <row r="56" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B56" s="7">
-        <v>57265</v>
+        <v>56489</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F56" s="9">
-        <v>1904612086</v>
+        <v>1608984973</v>
       </c>
       <c r="G56" s="10"/>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B57" s="7">
-        <v>57333</v>
+        <v>50328</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F57" s="9">
-        <v>1918352465</v>
+        <v>1608985572</v>
       </c>
       <c r="G57" s="10"/>
     </row>
     <row r="58" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B58" s="7">
-        <v>50328</v>
+        <v>40660</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F58" s="9">
-        <v>1608985572</v>
+        <v>1678863894</v>
       </c>
       <c r="G58" s="10"/>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B59" s="7">
-        <v>40660</v>
+        <v>42692</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F59" s="9">
-        <v>1678863894</v>
+        <v>1796322838</v>
       </c>
       <c r="G59" s="10"/>
     </row>
     <row r="60" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B60" s="7">
-        <v>42692</v>
+        <v>43264</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F60" s="9">
-        <v>1796322838</v>
+        <v>1722825343</v>
       </c>
       <c r="G60" s="10"/>
     </row>
     <row r="61" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B61" s="7">
-        <v>43264</v>
+        <v>57041</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F61" s="9">
-        <v>1722825343</v>
+        <v>1633794821</v>
       </c>
       <c r="G61" s="10"/>
     </row>
     <row r="62" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B62" s="7">
-        <v>57041</v>
+        <v>41904</v>
       </c>
       <c r="C62" s="8" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="E62" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F62" s="9">
-        <v>1633794821</v>
+        <v>1678862349</v>
       </c>
       <c r="G62" s="10"/>
     </row>
     <row r="63" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B63" s="7">
-        <v>41904</v>
+        <v>43249</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F63" s="9">
-        <v>1678862349</v>
+        <v>1817270543</v>
       </c>
       <c r="G63" s="10"/>
     </row>
     <row r="64" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B64" s="7">
-        <v>43249</v>
+        <v>60321</v>
       </c>
       <c r="C64" s="8" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E64" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F64" s="9">
-        <v>1817270543</v>
+        <v>1787803439</v>
       </c>
       <c r="G64" s="10"/>
     </row>
     <row r="65" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B65" s="7">
-        <v>60321</v>
+        <v>57208</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F65" s="9">
-        <v>1787803439</v>
+        <v>1633794809</v>
       </c>
       <c r="G65" s="10"/>
     </row>
     <row r="66" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B66" s="7">
-        <v>57208</v>
+        <v>60578</v>
       </c>
       <c r="C66" s="8" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F66" s="9">
-        <v>1633794809</v>
+        <v>1608984685</v>
       </c>
       <c r="G66" s="10"/>
     </row>
     <row r="67" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B67" s="7">
-        <v>60578</v>
+        <v>60586</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F67" s="9">
-        <v>1608984685</v>
+        <v>1633794820</v>
       </c>
       <c r="G67" s="10"/>
     </row>
     <row r="68" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B68" s="7">
-        <v>60586</v>
+        <v>60914</v>
       </c>
       <c r="C68" s="8" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E68" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F68" s="9">
-        <v>1633794820</v>
+        <v>1633794603</v>
       </c>
       <c r="G68" s="10"/>
     </row>
     <row r="69" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B69" s="7">
-        <v>60914</v>
+        <v>61071</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F69" s="9">
-        <v>1633794603</v>
+        <v>1608984563</v>
       </c>
       <c r="G69" s="10"/>
     </row>
     <row r="70" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B70" s="7">
-        <v>61071</v>
+        <v>61650</v>
       </c>
       <c r="C70" s="8" t="s">
-        <v>136</v>
+        <v>117</v>
       </c>
       <c r="D70" s="8" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E70" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F70" s="9">
-        <v>1608984563</v>
+        <v>1678860704</v>
       </c>
       <c r="G70" s="10"/>
     </row>
     <row r="71" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B71" s="7">
-        <v>61650</v>
+        <v>61674</v>
       </c>
       <c r="C71" s="8" t="s">
         <v>127</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F71" s="9">
-        <v>1678860704</v>
+        <v>1608984733</v>
       </c>
       <c r="G71" s="10"/>
     </row>
     <row r="72" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B72" s="7">
-        <v>61674</v>
+        <v>62193</v>
       </c>
       <c r="C72" s="8" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F72" s="9">
-        <v>1608984733</v>
+        <v>1678862208</v>
       </c>
       <c r="G72" s="10"/>
     </row>
     <row r="73" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B73" s="7">
-        <v>62193</v>
+        <v>62536</v>
       </c>
       <c r="C73" s="8" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F73" s="9">
-        <v>1678862208</v>
+        <v>1633794887</v>
       </c>
       <c r="G73" s="10"/>
     </row>
     <row r="74" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B74" s="7">
-        <v>62536</v>
+        <v>63089</v>
       </c>
       <c r="C74" s="8" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E74" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F74" s="9">
-        <v>1633794887</v>
+        <v>1633794814</v>
       </c>
       <c r="G74" s="10"/>
     </row>
     <row r="75" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B75" s="7">
-        <v>63089</v>
+        <v>63107</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="D75" s="8" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F75" s="9">
-        <v>1633794814</v>
+        <v>1633794845</v>
       </c>
       <c r="G75" s="10"/>
     </row>
     <row r="76" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B76" s="7">
-        <v>63107</v>
+        <v>63137</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="D76" s="8" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E76" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F76" s="9">
-        <v>1633794845</v>
+        <v>1633794844</v>
       </c>
       <c r="G76" s="10"/>
     </row>
     <row r="77" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B77" s="7">
-        <v>63137</v>
+        <v>63195</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="D77" s="8" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E77" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F77" s="9">
-        <v>1633794844</v>
+        <v>1633794471</v>
       </c>
       <c r="G77" s="10"/>
     </row>
     <row r="78" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B78" s="7">
-        <v>63195</v>
+        <v>63513</v>
       </c>
       <c r="C78" s="8" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="D78" s="8" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E78" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F78" s="9">
-        <v>1633794471</v>
+        <v>1608985910</v>
       </c>
       <c r="G78" s="10"/>
     </row>
     <row r="79" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B79" s="7">
-        <v>63513</v>
+        <v>65683</v>
       </c>
       <c r="C79" s="8" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="D79" s="8" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E79" s="8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="F79" s="9">
-        <v>1608985910</v>
+        <v>1633794808</v>
       </c>
       <c r="G79" s="10"/>
     </row>
-    <row r="80" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B80" s="7">
-        <v>64456</v>
-      </c>
-      <c r="C80" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="D80" s="8" t="s">
-        <v>132</v>
+    <row r="80" spans="2:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B80" s="11">
+        <v>63124</v>
+      </c>
+      <c r="C80" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="D80" s="12" t="s">
+        <v>137</v>
       </c>
       <c r="E80" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="F80" s="9">
-        <v>1633794867</v>
-      </c>
-      <c r="G80" s="10"/>
-    </row>
-    <row r="81" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B81" s="7">
-        <v>65683</v>
-      </c>
-      <c r="C81" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="D81" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="E81" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="F81" s="9">
-        <v>1633794808</v>
-      </c>
-      <c r="G81" s="10"/>
-    </row>
-    <row r="82" spans="2:7" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B82" s="11">
-        <v>63124</v>
-      </c>
-      <c r="C82" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="D82" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="E82" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="F82" s="13">
+        <v>145</v>
+      </c>
+      <c r="F80" s="13">
         <v>1761264863</v>
       </c>
-      <c r="G82" s="14"/>
+      <c r="G80" s="14"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{46A536A4-6FC6-4B68-9B3A-ECD9ADA4BF09}"/>
+    <hyperlink ref="G4" r:id="rId1" xr:uid="{46A536A4-6FC6-4B68-9B3A-ECD9ADA4BF09}"/>
+    <hyperlink ref="G29" r:id="rId2" xr:uid="{E63B8B4B-ADA7-449D-B7D4-1FE7CF5435BE}"/>
+    <hyperlink ref="G30" r:id="rId3" xr:uid="{7A5C5413-DD04-44FC-A2A5-CAE874C5DA65}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>